<commit_message>
commit updates on tracker
</commit_message>
<xml_diff>
--- a/modules/tracker/docs/templates/Question_Mapping.xlsx
+++ b/modules/tracker/docs/templates/Question_Mapping.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
   <si>
     <t xml:space="preserve">TURAS Tracker - Question Mapping</t>
   </si>
   <si>
-    <t xml:space="preserve">Map canonical question codes to actual column names in each wave's data file. Add wave columns (W4, W5, ...) as needed.</t>
+    <t xml:space="preserve">Map canonical question codes to actual column names in each wave's data file. Add more wave columns (W5, W6, ...) as needed.</t>
   </si>
   <si>
     <t xml:space="preserve">QuestionCode</t>
@@ -38,16 +38,25 @@
     <t xml:space="preserve">W3</t>
   </si>
   <si>
+    <t xml:space="preserve">W4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResponseScale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ScalePoints</t>
+  </si>
+  <si>
     <t xml:space="preserve">SourceQuestions</t>
   </si>
   <si>
     <t xml:space="preserve">TrackingSpecs</t>
   </si>
   <si>
-    <t xml:space="preserve">[REQUIRED] Canonical question code used across the tracking study</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Optional] Question text for documentation and report labels</t>
+    <t xml:space="preserve">[REQUIRED] Canonical question code used across the tracking study (must match TrackedQuestions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] Full question wording for documentation and report labels</t>
   </si>
   <si>
     <t xml:space="preserve">[Optional] Type of question for calculation method selection</t>
@@ -62,10 +71,19 @@
     <t xml:space="preserve">[Optional] Column name in Wave 3 data file for this question</t>
   </si>
   <si>
-    <t xml:space="preserve">[Optional] For Composite type: semicolon-separated list of source question columns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Optional] Comma-separated metrics to calculate: mean, top_box, top2_box, top3_box, bottom_box, bottom2_box, distribution, nps_score, promoters_pct, passives_pct, detractors_pct, full, all, auto, count_mean, range:X-Y, category:X, option:X</t>
+    <t xml:space="preserve">[Optional] Column name in Wave 4 data file for this question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] Scale description for documentation (e.g., '1=Very Dissatisfied to 5=Very Satisfied')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] Number of scale points for rating questions (e.g., 5, 7, 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] For Composite type: semicolon-separated list of source question codes that form the index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Optional] Comma-separated metrics (legacy location; prefer TrackedQuestions sheet). Specs: mean, top_box, top2_box, top3_box, bottom_box, bottom2_box, bottom3_box, distribution, nps_score, promoters_pct, passives_pct, detractors_pct, full, all, auto, count_mean, count_distribution, range:X-Y, box:CATEGORY, category:X, option:X</t>
   </si>
   <si>
     <t xml:space="preserve">Q01_Awareness</t>
@@ -86,6 +104,9 @@
     <t xml:space="preserve">Q15</t>
   </si>
   <si>
+    <t xml:space="preserve">Yes / No / Not sure</t>
+  </si>
+  <si>
     <t xml:space="preserve"/>
   </si>
   <si>
@@ -95,7 +116,7 @@
     <t xml:space="preserve">Q02_Satisfaction</t>
   </si>
   <si>
-    <t xml:space="preserve">Overall Satisfaction</t>
+    <t xml:space="preserve">Overall Satisfaction (1-10)</t>
   </si>
   <si>
     <t xml:space="preserve">Rating</t>
@@ -110,13 +131,16 @@
     <t xml:space="preserve">Q25</t>
   </si>
   <si>
+    <t xml:space="preserve">1=Very Dissatisfied to 10=Very Satisfied</t>
+  </si>
+  <si>
     <t xml:space="preserve">mean,top2_box</t>
   </si>
   <si>
     <t xml:space="preserve">Q03_NPS</t>
   </si>
   <si>
-    <t xml:space="preserve">Net Promoter Score</t>
+    <t xml:space="preserve">How likely to recommend? (0-10)</t>
   </si>
   <si>
     <t xml:space="preserve">NPS</t>
@@ -131,13 +155,16 @@
     <t xml:space="preserve">Q35</t>
   </si>
   <si>
-    <t xml:space="preserve">nps_score</t>
+    <t xml:space="preserve">0=Not at all likely to 10=Extremely likely</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nps_score,promoters_pct,detractors_pct</t>
   </si>
   <si>
     <t xml:space="preserve">Q04_Purchase</t>
   </si>
   <si>
-    <t xml:space="preserve">Purchase Intent</t>
+    <t xml:space="preserve">How likely to purchase?</t>
   </si>
   <si>
     <t xml:space="preserve">Q40</t>
@@ -149,13 +176,16 @@
     <t xml:space="preserve">Q45</t>
   </si>
   <si>
-    <t xml:space="preserve">top_box</t>
+    <t xml:space="preserve">Definitely / Probably / Might / Probably Not / Definitely Not</t>
+  </si>
+  <si>
+    <t xml:space="preserve">category:Definitely</t>
   </si>
   <si>
     <t xml:space="preserve">Q05_Features</t>
   </si>
   <si>
-    <t xml:space="preserve">Features Used</t>
+    <t xml:space="preserve">Which features have you used?</t>
   </si>
   <si>
     <t xml:space="preserve">Multi_Mention</t>
@@ -170,10 +200,52 @@
     <t xml:space="preserve">Q55</t>
   </si>
   <si>
+    <t xml:space="preserve">Select all that apply</t>
+  </si>
+  <si>
     <t xml:space="preserve">Q50_1;Q50_2;Q50_3</t>
   </si>
   <si>
     <t xml:space="preserve">auto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q06_Agreement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service meets expectations (1-5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q62</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1=Strongly Disagree to 5=Strongly Agree</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean,box:Agree=Top Box</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q07_CX_Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Experience Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculated index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q02_Satisfaction;Q06_Agreement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean</t>
   </si>
 </sst>
 </file>
@@ -608,8 +680,11 @@
     <col min="4" max="4" width="18.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="18.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="30.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="40.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="18.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="25.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="14.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="30.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="40.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -647,182 +722,295 @@
       <c r="H3" s="3" t="s">
         <v>9</v>
       </c>
+      <c r="I3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>17</v>
+        <v>20</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>25</v>
+        <v>30</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>32</v>
+      <c r="K6" s="5" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>39</v>
+        <v>47</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>53</v>
+        <v>62</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
+      <c r="A10" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
+      <c r="A11" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6"/>
@@ -833,6 +1021,9 @@
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
     </row>
     <row r="13">
       <c r="A13" s="6"/>
@@ -843,6 +1034,9 @@
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
     </row>
     <row r="14">
       <c r="A14" s="6"/>
@@ -853,6 +1047,9 @@
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
     </row>
     <row r="15">
       <c r="A15" s="6"/>
@@ -863,6 +1060,9 @@
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
     </row>
     <row r="16">
       <c r="A16" s="6"/>
@@ -873,6 +1073,9 @@
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
     </row>
     <row r="17">
       <c r="A17" s="6"/>
@@ -883,6 +1086,9 @@
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
     </row>
     <row r="18">
       <c r="A18" s="6"/>
@@ -893,6 +1099,9 @@
       <c r="F18" s="6"/>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
     </row>
     <row r="19">
       <c r="A19" s="6"/>
@@ -903,6 +1112,9 @@
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
     </row>
     <row r="20">
       <c r="A20" s="6"/>
@@ -913,6 +1125,9 @@
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
     </row>
     <row r="21">
       <c r="A21" s="6"/>
@@ -923,6 +1138,9 @@
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
     </row>
     <row r="22">
       <c r="A22" s="6"/>
@@ -933,6 +1151,9 @@
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
     </row>
     <row r="23">
       <c r="A23" s="6"/>
@@ -943,6 +1164,9 @@
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
     </row>
     <row r="24">
       <c r="A24" s="6"/>
@@ -953,6 +1177,9 @@
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
     </row>
     <row r="25">
       <c r="A25" s="6"/>
@@ -963,6 +1190,9 @@
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
     </row>
     <row r="26">
       <c r="A26" s="6"/>
@@ -973,6 +1203,9 @@
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
     </row>
     <row r="27">
       <c r="A27" s="6"/>
@@ -983,6 +1216,9 @@
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
     </row>
     <row r="28">
       <c r="A28" s="6"/>
@@ -993,6 +1229,9 @@
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
     </row>
     <row r="29">
       <c r="A29" s="6"/>
@@ -1003,6 +1242,9 @@
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
     </row>
     <row r="30">
       <c r="A30" s="6"/>
@@ -1013,6 +1255,9 @@
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
+      <c r="I30" s="6"/>
+      <c r="J30" s="6"/>
+      <c r="K30" s="6"/>
     </row>
     <row r="31">
       <c r="A31" s="6"/>
@@ -1023,6 +1268,9 @@
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
     </row>
     <row r="32">
       <c r="A32" s="6"/>
@@ -1033,6 +1281,9 @@
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
     </row>
     <row r="33">
       <c r="A33" s="6"/>
@@ -1043,6 +1294,9 @@
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6"/>
+      <c r="K33" s="6"/>
     </row>
     <row r="34">
       <c r="A34" s="6"/>
@@ -1053,6 +1307,9 @@
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="6"/>
     </row>
     <row r="35">
       <c r="A35" s="6"/>
@@ -1063,6 +1320,9 @@
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="6"/>
+      <c r="K35" s="6"/>
     </row>
     <row r="36">
       <c r="A36" s="6"/>
@@ -1073,6 +1333,9 @@
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
     </row>
     <row r="37">
       <c r="A37" s="6"/>
@@ -1083,6 +1346,9 @@
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
     </row>
     <row r="38">
       <c r="A38" s="6"/>
@@ -1093,6 +1359,9 @@
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
+      <c r="I38" s="6"/>
+      <c r="J38" s="6"/>
+      <c r="K38" s="6"/>
     </row>
     <row r="39">
       <c r="A39" s="6"/>
@@ -1103,6 +1372,9 @@
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="6"/>
+      <c r="K39" s="6"/>
     </row>
     <row r="40">
       <c r="A40" s="6"/>
@@ -1113,6 +1385,9 @@
       <c r="F40" s="6"/>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
+      <c r="I40" s="6"/>
+      <c r="J40" s="6"/>
+      <c r="K40" s="6"/>
     </row>
     <row r="41">
       <c r="A41" s="6"/>
@@ -1123,6 +1398,9 @@
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
+      <c r="I41" s="6"/>
+      <c r="J41" s="6"/>
+      <c r="K41" s="6"/>
     </row>
     <row r="42">
       <c r="A42" s="6"/>
@@ -1133,6 +1411,9 @@
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="6"/>
+      <c r="K42" s="6"/>
     </row>
     <row r="43">
       <c r="A43" s="6"/>
@@ -1143,6 +1424,9 @@
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6"/>
     </row>
     <row r="44">
       <c r="A44" s="6"/>
@@ -1153,6 +1437,9 @@
       <c r="F44" s="6"/>
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6"/>
     </row>
     <row r="45">
       <c r="A45" s="6"/>
@@ -1163,6 +1450,9 @@
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
+      <c r="I45" s="6"/>
+      <c r="J45" s="6"/>
+      <c r="K45" s="6"/>
     </row>
     <row r="46">
       <c r="A46" s="6"/>
@@ -1173,6 +1463,9 @@
       <c r="F46" s="6"/>
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
+      <c r="I46" s="6"/>
+      <c r="J46" s="6"/>
+      <c r="K46" s="6"/>
     </row>
     <row r="47">
       <c r="A47" s="6"/>
@@ -1183,6 +1476,9 @@
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
+      <c r="I47" s="6"/>
+      <c r="J47" s="6"/>
+      <c r="K47" s="6"/>
     </row>
     <row r="48">
       <c r="A48" s="6"/>
@@ -1193,6 +1489,9 @@
       <c r="F48" s="6"/>
       <c r="G48" s="6"/>
       <c r="H48" s="6"/>
+      <c r="I48" s="6"/>
+      <c r="J48" s="6"/>
+      <c r="K48" s="6"/>
     </row>
     <row r="49">
       <c r="A49" s="6"/>
@@ -1203,6 +1502,9 @@
       <c r="F49" s="6"/>
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6"/>
+      <c r="K49" s="6"/>
     </row>
     <row r="50">
       <c r="A50" s="6"/>
@@ -1213,6 +1515,9 @@
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
       <c r="H50" s="6"/>
+      <c r="I50" s="6"/>
+      <c r="J50" s="6"/>
+      <c r="K50" s="6"/>
     </row>
     <row r="51">
       <c r="A51" s="6"/>
@@ -1223,6 +1528,9 @@
       <c r="F51" s="6"/>
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
+      <c r="I51" s="6"/>
+      <c r="J51" s="6"/>
+      <c r="K51" s="6"/>
     </row>
     <row r="52">
       <c r="A52" s="6"/>
@@ -1233,6 +1541,9 @@
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
       <c r="H52" s="6"/>
+      <c r="I52" s="6"/>
+      <c r="J52" s="6"/>
+      <c r="K52" s="6"/>
     </row>
     <row r="53">
       <c r="A53" s="6"/>
@@ -1243,6 +1554,9 @@
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
     </row>
     <row r="54">
       <c r="A54" s="6"/>
@@ -1253,6 +1567,9 @@
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
+      <c r="I54" s="6"/>
+      <c r="J54" s="6"/>
+      <c r="K54" s="6"/>
     </row>
     <row r="55">
       <c r="A55" s="6"/>
@@ -1263,6 +1580,9 @@
       <c r="F55" s="6"/>
       <c r="G55" s="6"/>
       <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6"/>
+      <c r="K55" s="6"/>
     </row>
     <row r="56">
       <c r="A56" s="6"/>
@@ -1273,6 +1593,9 @@
       <c r="F56" s="6"/>
       <c r="G56" s="6"/>
       <c r="H56" s="6"/>
+      <c r="I56" s="6"/>
+      <c r="J56" s="6"/>
+      <c r="K56" s="6"/>
     </row>
     <row r="57">
       <c r="A57" s="6"/>
@@ -1283,6 +1606,9 @@
       <c r="F57" s="6"/>
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
+      <c r="I57" s="6"/>
+      <c r="J57" s="6"/>
+      <c r="K57" s="6"/>
     </row>
     <row r="58">
       <c r="A58" s="6"/>
@@ -1293,6 +1619,9 @@
       <c r="F58" s="6"/>
       <c r="G58" s="6"/>
       <c r="H58" s="6"/>
+      <c r="I58" s="6"/>
+      <c r="J58" s="6"/>
+      <c r="K58" s="6"/>
     </row>
     <row r="59">
       <c r="A59" s="6"/>
@@ -1303,12 +1632,47 @@
       <c r="F59" s="6"/>
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
+      <c r="I59" s="6"/>
+      <c r="J59" s="6"/>
+      <c r="K59" s="6"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6"/>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="6"/>
+      <c r="H60" s="6"/>
+      <c r="I60" s="6"/>
+      <c r="J60" s="6"/>
+      <c r="K60" s="6"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6"/>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6"/>
+      <c r="H61" s="6"/>
+      <c r="I61" s="6"/>
+      <c r="J61" s="6"/>
+      <c r="K61" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="whole" operator="between" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I61">
+      <formula1>2</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <extLst>
@@ -1318,7 +1682,7 @@
           <x14:formula1>
             <xm:f>"Rating,NPS,Single_Response,Multi_Mention,Composite"</xm:f>
           </x14:formula1>
-          <xm:sqref>C5:C59</xm:sqref>
+          <xm:sqref>C5:C61</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>